<commit_message>
Uopdated hitscan and excel
</commit_message>
<xml_diff>
--- a/Other/Book1.xlsx
+++ b/Other/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\U2260777\Downloads\DisertationWork\Other\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F485F754-2327-45BC-B721-52C14C593F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10423260-2023-41BF-90FC-5BD7107B2575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{F69A984C-CCA6-4246-82C5-767B2FF15A7B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="14">
   <si>
     <t>None</t>
   </si>
@@ -75,13 +75,16 @@
   </si>
   <si>
     <t>Music Sound Test</t>
+  </si>
+  <si>
+    <t>Time</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -110,8 +113,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -128,6 +138,11 @@
         <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -138,19 +153,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="3"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
+    <cellStyle name="Good" xfId="3" builtinId="26"/>
     <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -485,22 +503,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27FF0422-255B-404C-AE6B-B5A828AC21C0}">
   <dimension ref="A13:Y83"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.5" customWidth="1"/>
-    <col min="3" max="3" width="17.625" customWidth="1"/>
-    <col min="4" max="4" width="17.5" customWidth="1"/>
-    <col min="5" max="5" width="16.625" customWidth="1"/>
-    <col min="6" max="6" width="24.75" customWidth="1"/>
-    <col min="22" max="22" width="10.5" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" customWidth="1"/>
+    <col min="3" max="3" width="17.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" customWidth="1"/>
+    <col min="6" max="6" width="24.7109375" customWidth="1"/>
+    <col min="22" max="22" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="13" spans="1:22" ht="36">
+    <row r="13" spans="1:22" ht="36" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:22">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -519,13 +537,16 @@
       <c r="F14" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="1:22">
+      <c r="G14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:22">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16">
         <f>A15+1</f>
         <v>2</v>
@@ -534,7 +555,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:25">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17">
         <f t="shared" ref="A17:A31" si="0">A16+1</f>
         <v>3</v>
@@ -542,7 +563,7 @@
       <c r="V17" s="2">
         <v>1</v>
       </c>
-      <c r="W17" s="1" t="s">
+      <c r="W17" s="4" t="s">
         <v>0</v>
       </c>
       <c r="X17" s="1" t="s">
@@ -552,7 +573,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:25">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -571,7 +592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:25">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -590,7 +611,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:25">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -609,7 +630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:25">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -628,7 +649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:25">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -647,7 +668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:25">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -666,7 +687,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:25">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A24">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -685,7 +706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:25">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -704,7 +725,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:25">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -723,7 +744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:25">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -742,7 +763,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:25">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -761,7 +782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:25">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -780,7 +801,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:25">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -799,7 +820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:25">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -818,7 +839,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:25">
+    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A32">
         <f>A31+1</f>
         <v>18</v>
@@ -837,7 +858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:25">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
       <c r="V33" s="1">
         <f t="shared" si="1"/>
         <v>17</v>
@@ -852,7 +873,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:25">
+    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
       <c r="V34" s="1">
         <f t="shared" si="1"/>
         <v>18</v>
@@ -867,12 +888,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:25" ht="36">
+    <row r="39" spans="1:25" ht="36" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:25">
+    <row r="40" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>4</v>
       </c>
@@ -891,120 +912,123 @@
       <c r="F40" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="41" spans="1:25">
+      <c r="G40" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:25">
+    <row r="42" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A42">
         <f>A41+1</f>
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="1:25">
+    <row r="43" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A43">
         <f t="shared" ref="A43:A57" si="2">A42+1</f>
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:25">
+    <row r="44" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A44">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:25">
+    <row r="45" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A45">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:25">
+    <row r="46" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A46">
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:25">
+    <row r="47" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A47">
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:25">
+    <row r="48" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A48">
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="1:1">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49">
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:1">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
     </row>
-    <row r="51" spans="1:1">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51">
         <f t="shared" si="2"/>
         <v>11</v>
       </c>
     </row>
-    <row r="52" spans="1:1">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52">
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
     </row>
-    <row r="53" spans="1:1">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53">
         <f t="shared" si="2"/>
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:1">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54">
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
     </row>
-    <row r="55" spans="1:1">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55">
         <f t="shared" si="2"/>
         <v>15</v>
       </c>
     </row>
-    <row r="56" spans="1:1">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56">
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
     </row>
-    <row r="57" spans="1:1">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57">
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
     </row>
-    <row r="58" spans="1:1">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58">
         <f>A57+1</f>
         <v>18</v>
       </c>
     </row>
-    <row r="64" spans="1:1" ht="36">
+    <row r="64" spans="1:1" ht="36" x14ac:dyDescent="0.55000000000000004">
       <c r="A64" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>4</v>
       </c>
@@ -1023,109 +1047,112 @@
       <c r="F65" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="66" spans="1:6">
+      <c r="G65" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67">
         <f>A66+1</f>
         <v>2</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68">
         <f t="shared" ref="A68:A82" si="3">A67+1</f>
         <v>3</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72">
         <f t="shared" si="3"/>
         <v>7</v>
       </c>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73">
         <f t="shared" si="3"/>
         <v>8</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74">
         <f t="shared" si="3"/>
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="1:6">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75">
         <f t="shared" si="3"/>
         <v>10</v>
       </c>
     </row>
-    <row r="76" spans="1:6">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76">
         <f t="shared" si="3"/>
         <v>11</v>
       </c>
     </row>
-    <row r="77" spans="1:6">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77">
         <f t="shared" si="3"/>
         <v>12</v>
       </c>
     </row>
-    <row r="78" spans="1:6">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78">
         <f t="shared" si="3"/>
         <v>13</v>
       </c>
     </row>
-    <row r="79" spans="1:6">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79">
         <f t="shared" si="3"/>
         <v>14</v>
       </c>
     </row>
-    <row r="80" spans="1:6">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80">
         <f t="shared" si="3"/>
         <v>15</v>
       </c>
     </row>
-    <row r="81" spans="1:1">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81">
         <f t="shared" si="3"/>
         <v>16</v>
       </c>
     </row>
-    <row r="82" spans="1:1">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82">
         <f t="shared" si="3"/>
         <v>17</v>
       </c>
     </row>
-    <row r="83" spans="1:1">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83">
         <f>A82+1</f>
         <v>18</v>

</xml_diff>